<commit_message>
feat: Rebrand to Suara Surabaya Media, 5-second login slider, light/dark mode, and cleanup
</commit_message>
<xml_diff>
--- a/MBKM1-10_3_Lembar_Pengujian_SAD.xlsx
+++ b/MBKM1-10_3_Lembar_Pengujian_SAD.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="401" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="392">
   <si>
     <t>Objektivitas</t>
   </si>
@@ -536,14 +536,671 @@
     <t>Proses ditingkatkan untuk Sprint berikutnya tetapi bisa memberatkan kinerja perseorangan</t>
   </si>
   <si>
+    <t>Dokumen SRS lengkap mencakup Use Case, Activity Diagram, dan ERD database PostgreSQL</t>
+  </si>
+  <si>
+    <t>Desain UI/UX mengikuti standar "Civic Flow" dari Google Stitch dengan palet warna Primary Blue (#1D4ED8) dan tipografi Inter/Plus Jakarta Sans</t>
+  </si>
+  <si>
+    <t>Sistem fullstack berjalan: Backend Laravel 11 (REST API) + Frontend Next.js 14 (TypeScript) + Database PostgreSQL + Supabase Storage</t>
+  </si>
+  <si>
+    <t>Seluruh fitur utama (Login, Registrasi, Pengajuan Magang, Review Dokumen, Algoritma DSS, Export Excel) diuji secara Blackbox dan Whitebox</t>
+  </si>
+  <si>
+    <t>Sistem berjalan di lingkungan lokal (Backend: localhost:8000, Frontend: localhost:3000)</t>
+  </si>
+  <si>
+    <t>Bug ditemukan dan diperbaiki selama sesi pengembangan secara iteratif</t>
+  </si>
+  <si>
     <t>Hasil yang Diharapkan</t>
+  </si>
+  <si>
+    <t>TC_LR_001</t>
+  </si>
+  <si>
+    <t>Login dengan kredensial valid (Admin)</t>
+  </si>
+  <si>
+    <t>Email: admin@dishub.go.id, Password: password</t>
+  </si>
+  <si>
+    <t>Berhasil masuk ke Dashboard Admin</t>
+  </si>
+  <si>
+    <t>Autentikasi via Laravel Sanctum berjalan normal</t>
+  </si>
+  <si>
+    <t>TC_LR_002</t>
+  </si>
+  <si>
+    <t>Login dengan kredensial valid (Pimpinan)</t>
+  </si>
+  <si>
+    <t>Email: head@dishub.go.id, Password: password</t>
+  </si>
+  <si>
+    <t>Berhasil masuk ke Dashboard Pimpinan</t>
+  </si>
+  <si>
+    <t>Routing berbasis role berfungsi</t>
+  </si>
+  <si>
+    <t>TC_LR_003</t>
+  </si>
+  <si>
+    <t>Login dengan kredensial tidak valid</t>
+  </si>
+  <si>
+    <t>Email: test@test.com, Password: salah</t>
+  </si>
+  <si>
+    <t>Muncul pesan error "Email atau password salah"</t>
+  </si>
+  <si>
+    <t>Validasi error ditampilkan dengan benar</t>
+  </si>
+  <si>
+    <t>TC_LR_004</t>
+  </si>
+  <si>
+    <t>Registrasi akun baru pelamar</t>
+  </si>
+  <si>
+    <t>Nama: Test User, Email: test@mail.com, Password: 12345678, Tipe: Mahasiswa</t>
+  </si>
+  <si>
+    <t>Akun berhasil dibuat dan redirect ke login</t>
+  </si>
+  <si>
+    <t>Registrasi menyimpan data ke database PostgreSQL</t>
+  </si>
+  <si>
+    <t>TC_PP_001</t>
+  </si>
+  <si>
+    <t>Pengajuan magang oleh pelamar</t>
+  </si>
+  <si>
+    <t>Divisi: Angkutan, Tanggal: 01/06/2026-01/09/2026, Upload CV + KTP + Surat Pengantar</t>
+  </si>
+  <si>
+    <t>Pengajuan tersimpan dengan status "Pending"</t>
+  </si>
+  <si>
+    <t>Dokumen terunggah ke Supabase Storage</t>
+  </si>
+  <si>
+    <t>TC_PP_002</t>
+  </si>
+  <si>
+    <t>Pelamar melihat status pengajuan</t>
+  </si>
+  <si>
+    <t>Login sebagai pelamar, akses halaman status</t>
+  </si>
+  <si>
+    <t>Menampilkan status pengajuan terkini</t>
+  </si>
+  <si>
+    <t>Menampilkan status pengajuan terkini beserta detail dokumen</t>
+  </si>
+  <si>
+    <t>Data konsisten dengan keputusan admin</t>
+  </si>
+  <si>
+    <t>TC_PP_003</t>
+  </si>
+  <si>
+    <t>Pelamar melihat notifikasi</t>
+  </si>
+  <si>
+    <t>Login sebagai pelamar, akses halaman notifikasi</t>
+  </si>
+  <si>
+    <t>Menampilkan daftar notifikasi terbaru</t>
+  </si>
+  <si>
+    <t>Notifikasi otomatis terkirim saat status berubah</t>
+  </si>
+  <si>
+    <t>TC_AA_001</t>
+  </si>
+  <si>
+    <t>Admin menjalankan algoritma sortir (DSS)</t>
+  </si>
+  <si>
+    <t>Klik tombol "Proses Algoritma" pada daftar pelamar</t>
+  </si>
+  <si>
+    <t>Sistem menampilkan hasil R1, R3, R4 dan skor algoritma</t>
+  </si>
+  <si>
+    <t>Decision Support System berjalan sesuai aturan bisnis</t>
+  </si>
+  <si>
+    <t>TC_AA_002</t>
+  </si>
+  <si>
+    <t>Admin menerima pengajuan pelamar</t>
+  </si>
+  <si>
+    <t>Klik "Terima" pada detail pelamar, tambahkan catatan admin</t>
+  </si>
+  <si>
+    <t>Status berubah menjadi "Diterima" dan notifikasi terkirim</t>
+  </si>
+  <si>
+    <t>Kuota divisi berkurang otomatis</t>
+  </si>
+  <si>
+    <t>TC_AA_003</t>
+  </si>
+  <si>
+    <t>Admin menolak pengajuan pelamar</t>
+  </si>
+  <si>
+    <t>Klik "Tolak", isi alasan penolakan</t>
+  </si>
+  <si>
+    <t>Status berubah menjadi "Ditolak" dengan alasan tersimpan</t>
+  </si>
+  <si>
+    <t>Notifikasi penolakan terkirim ke pelamar</t>
+  </si>
+  <si>
+    <t>TC_AA_004</t>
+  </si>
+  <si>
+    <t>Admin menekan tombol "Lihat Dokumen" (Percobaan Pertama - GAGAL)</t>
+  </si>
+  <si>
+    <t>Klik ikon mata pada baris dokumen CV pelamar</t>
+  </si>
+  <si>
+    <t>Muncul pop-up preview menampilkan file PDF</t>
+  </si>
+  <si>
+    <t>Pop-up terbuka tetapi menampilkan error "404 - This page could not be found"</t>
+  </si>
+  <si>
+    <t>Iframe memanggil relative path database mentah (documents/123_cv.pdf) bukan URL absolut Supabase</t>
+  </si>
+  <si>
+    <t>TC_AA_005</t>
+  </si>
+  <si>
+    <t>Admin menekan tombol "Lihat Dokumen" (Percobaan Kedua - BERHASIL)</t>
+  </si>
+  <si>
+    <t>Pop-up terbuka dan file PDF berhasil ditampilkan di dalam iframe</t>
+  </si>
+  <si>
+    <t>Setelah perbaikan Accessor getFileUrlAttribute di Model Document.php, URL menjadi absolut</t>
+  </si>
+  <si>
+    <t>TC_AA_006</t>
+  </si>
+  <si>
+    <t>Admin mengelola divisi (Tambah)</t>
+  </si>
+  <si>
+    <t>Nama: Divisi Baru, Kuota: 10</t>
+  </si>
+  <si>
+    <t>Divisi berhasil ditambahkan</t>
+  </si>
+  <si>
+    <t>Data tersimpan di tabel divisions</t>
+  </si>
+  <si>
+    <t>TC_AA_007</t>
+  </si>
+  <si>
+    <t>Admin mengunci divisi</t>
+  </si>
+  <si>
+    <t>Klik tombol kunci pada divisi tertentu</t>
+  </si>
+  <si>
+    <t>Divisi terkunci dan tidak menerima pelamar baru</t>
+  </si>
+  <si>
+    <t>Field is_locked berubah menjadi true</t>
+  </si>
+  <si>
+    <t>TC_AP_001</t>
+  </si>
+  <si>
+    <t>Pimpinan melihat dashboard analitik</t>
+  </si>
+  <si>
+    <t>Login sebagai Pimpinan, akses halaman Dashboard</t>
+  </si>
+  <si>
+    <t>Menampilkan statistik: total pelamar, diterima, ditolak, grafik</t>
+  </si>
+  <si>
+    <t>Data real-time dari API analytics</t>
+  </si>
+  <si>
+    <t>TC_AP_002</t>
+  </si>
+  <si>
+    <t>Pimpinan menekan tombol Refresh</t>
+  </si>
+  <si>
+    <t>Klik tombol "Refresh" di dashboard</t>
+  </si>
+  <si>
+    <t>Data analitik diperbarui tanpa reload halaman</t>
+  </si>
+  <si>
+    <t>Data analitik diperbarui tanpa reload halaman dengan animasi loading</t>
+  </si>
+  <si>
+    <t>Tombol refresh berhasil ditambahkan dan berfungsi</t>
+  </si>
+  <si>
+    <t>TC_AP_003</t>
+  </si>
+  <si>
+    <t>Pimpinan mengekspor Excel (Percobaan Pertama - GAGAL)</t>
+  </si>
+  <si>
+    <t>Klik "Ekspor ke Excel" tanpa filter</t>
+  </si>
+  <si>
+    <t>File .xlsx terunduh otomatis</t>
+  </si>
+  <si>
+    <t>Muncul toast error: "Gagal mengunggah file export: 415 invalid_mime_type"</t>
+  </si>
+  <si>
+    <t>Supabase Storage menolak MIME type application/vnd.openxmlformats-officedocument.spreadsheetml.sheet</t>
+  </si>
+  <si>
+    <t>TC_AP_004</t>
+  </si>
+  <si>
+    <t>Pimpinan mengekspor Excel (Percobaan Kedua - GAGAL)</t>
+  </si>
+  <si>
+    <t>Klik "Ekspor ke Excel" setelah bypass Supabase</t>
+  </si>
+  <si>
+    <t>Muncul error HTTP 500: "Return value must be of type JsonResponse, BinaryFileResponse returned"</t>
+  </si>
+  <si>
+    <t>Konflik strict typing PHP 8 pada return type fungsi export() di HeadController</t>
+  </si>
+  <si>
+    <t>TC_AP_005</t>
+  </si>
+  <si>
+    <t>Pimpinan mengekspor Excel (Percobaan Ketiga - BERHASIL)</t>
+  </si>
+  <si>
+    <t>File Laporan_Magang_*.xlsx berhasil terunduh ke perangkat</t>
+  </si>
+  <si>
+    <t>Setelah perbaikan return type dan penambahan responseType blob di frontend</t>
+  </si>
+  <si>
+    <t>TC_AP_006</t>
+  </si>
+  <si>
+    <t>Pimpinan mengekspor Excel dengan filter</t>
+  </si>
+  <si>
+    <t>Filter: Status=Diterima, Divisi=Angkutan</t>
+  </si>
+  <si>
+    <t>File .xlsx terunduh dengan data terfilter</t>
+  </si>
+  <si>
+    <t>File .xlsx terunduh dengan data sesuai filter</t>
+  </si>
+  <si>
+    <t>Filter berfungsi pada query database</t>
+  </si>
+  <si>
+    <t>Menguji Accessor getFileUrlAttribute() dengan file_path valid</t>
+  </si>
+  <si>
+    <t>Document::getFileUrlAttribute() di backend/app/Models/Document.php</t>
+  </si>
+  <si>
+    <t>file_path: "applications/1/cv/resume.pdf"</t>
+  </si>
+  <si>
+    <t>Mengembalikan URL absolut Supabase: https://xxx.supabase.co/storage/v1/object/public/e-internship-documents/applications/1/cv/resume.pdf</t>
+  </si>
+  <si>
+    <t>Mengembalikan URL absolut Supabase yang valid</t>
+  </si>
+  <si>
+    <t>Baris 18-26 dieksekusi (Accessor + getPublicUrl)</t>
+  </si>
+  <si>
+    <t>Path relatif berhasil dikonversi ke Public URL</t>
+  </si>
+  <si>
+    <t>Menguji Accessor getFileUrlAttribute() dengan file_path null</t>
+  </si>
+  <si>
+    <t>file_path: null</t>
+  </si>
+  <si>
+    <t>Mengembalikan null</t>
+  </si>
+  <si>
+    <t>Baris 18-20 dieksekusi (early return)</t>
+  </si>
+  <si>
+    <t>Penanganan null berfungsi</t>
+  </si>
+  <si>
+    <t>Menguji Accessor getFileUrlAttribute() dengan URL http lengkap</t>
+  </si>
+  <si>
+    <t>file_path: "https://example.com/file.pdf"</t>
+  </si>
+  <si>
+    <t>Mengembalikan URL asli tanpa modifikasi</t>
+  </si>
+  <si>
+    <t>Baris 18-22 dieksekusi (str_starts_with check)</t>
+  </si>
+  <si>
+    <t>URL yang sudah absolut tidak di-double prefix</t>
+  </si>
+  <si>
+    <t>Menguji fungsi export() dengan upload ke Supabase (Percobaan Pertama - GAGAL)</t>
+  </si>
+  <si>
+    <t>HeadController::export() dengan $this-&gt;storage-&gt;uploadRaw()</t>
+  </si>
+  <si>
+    <t>Filter kosong (semua data)</t>
+  </si>
+  <si>
+    <t>File .xlsx terunggah ke Supabase dan URL download dikembalikan</t>
+  </si>
+  <si>
+    <t>Exception thrown: 415 invalid_mime_type dari Supabase API</t>
+  </si>
+  <si>
+    <t>Baris 230-239 dieksekusi (uploadRaw gagal, masuk catch block)</t>
+  </si>
+  <si>
+    <t>Supabase Bucket Policy memblokir MIME type .xlsx secara default</t>
+  </si>
+  <si>
+    <t>Menguji fungsi export() dengan return type JsonResponse (Percobaan Kedua - GAGAL)</t>
+  </si>
+  <si>
+    <t>HeadController::export(): JsonResponse dengan response()-&gt;download()</t>
+  </si>
+  <si>
+    <t>File .xlsx di-stream langsung ke browser</t>
+  </si>
+  <si>
+    <t>PHP Fatal Error: Return value must be of type JsonResponse, BinaryFileResponse returned</t>
+  </si>
+  <si>
+    <t>Baris 102 (deklarasi fungsi) menyebabkan TypeError</t>
+  </si>
+  <si>
+    <t>Strict typing PHP 8 menolak BinaryFileResponse saat deklarasi memaksakan JsonResponse</t>
+  </si>
+  <si>
+    <t>Menguji fungsi export() dengan union return type (Percobaan Ketiga - BERHASIL)</t>
+  </si>
+  <si>
+    <t>HeadController::export(): BinaryFileResponse|JsonResponse</t>
+  </si>
+  <si>
+    <t>File .xlsx di-stream langsung ke browser sebagai download</t>
+  </si>
+  <si>
+    <t>File .xlsx berhasil di-generate dan dikirim sebagai HTTP binary stream</t>
+  </si>
+  <si>
+    <t>Baris 102, 223-233 dieksekusi (Xlsx save + response download + deleteFileAfterSend)</t>
+  </si>
+  <si>
+    <t>Bypass Supabase + Union type PHP berhasil menyelesaikan kedua error</t>
+  </si>
+  <si>
+    <t>TC_WB_007</t>
+  </si>
+  <si>
+    <t>Menguji algoritma sortir R1 (Kelengkapan Dokumen)</t>
+  </si>
+  <si>
+    <t>AlgorithmService::checkR1()</t>
+  </si>
+  <si>
+    <t>Application dengan 3 dokumen lengkap (CV, KTP, Surat Pengantar)</t>
+  </si>
+  <si>
+    <t>r1_passed = true</t>
+  </si>
+  <si>
+    <t>Seluruh validasi dokumen dieksekusi</t>
+  </si>
+  <si>
+    <t>Validasi kelengkapan dokumen berfungsi</t>
+  </si>
+  <si>
+    <t>TC_WB_008</t>
+  </si>
+  <si>
+    <t>Menguji algoritma sortir R3 (Ketersediaan Kuota)</t>
+  </si>
+  <si>
+    <t>AlgorithmService::checkR3()</t>
+  </si>
+  <si>
+    <t>Division dengan max_quota=10, active_applicants=9</t>
+  </si>
+  <si>
+    <t>r3_passed = true (masih tersedia 1 slot)</t>
+  </si>
+  <si>
+    <t>r3_passed = true</t>
+  </si>
+  <si>
+    <t>Perbandingan kuota dieksekusi</t>
+  </si>
+  <si>
+    <t>Pengecekan kuota divisi berfungsi</t>
+  </si>
+  <si>
+    <t>TC_WB_009</t>
+  </si>
+  <si>
+    <t>Menguji algoritma sortir R4 (Keyword Matching)</t>
+  </si>
+  <si>
+    <t>AlgorithmService::checkR4()</t>
+  </si>
+  <si>
+    <t>study_program: "Teknik Informatika", division keywords: ["informatika", "teknologi"]</t>
+  </si>
+  <si>
+    <t>r4_passed = true, algorithm_score &gt; 60</t>
+  </si>
+  <si>
+    <t>r4_passed = true, algorithm_score = 75.5</t>
+  </si>
+  <si>
+    <t>Seluruh logika string matching dieksekusi</t>
+  </si>
+  <si>
+    <t>Keyword matching menghitung skor kesesuaian dengan benar</t>
+  </si>
+  <si>
+    <t>TC_WB_010</t>
+  </si>
+  <si>
+    <t>Menguji middleware RoleMiddleware untuk otorisasi</t>
+  </si>
+  <si>
+    <t>RoleMiddleware::handle()</t>
+  </si>
+  <si>
+    <t>User dengan role "applicant" mengakses route /admin/*</t>
+  </si>
+  <si>
+    <t>Response 403 Forbidden</t>
+  </si>
+  <si>
+    <t>Baris pengecekan role dan abort(403) dieksekusi</t>
+  </si>
+  <si>
+    <t>Middleware mencegah akses tidak sah ke panel admin</t>
+  </si>
+  <si>
+    <t>Dokumen SRS lengkap mencakup Use Case, Activity Diagram, dan ERD</t>
+  </si>
+  <si>
+    <t>Dokumen kebutuhan terstruktur dan dapat dijadikan acuan pengembangan</t>
+  </si>
+  <si>
+    <t>SRS telah mencakup ERD PostgreSQL (7 tabel), Use Case 3 aktor, dan Activity Diagram</t>
+  </si>
+  <si>
+    <t>Desain mengikuti standar "Civic Flow" dengan Primary Blue dan tipografi Inter</t>
+  </si>
+  <si>
+    <t>Antarmuka modern, konsisten, dan responsif di semua halaman</t>
+  </si>
+  <si>
+    <t>Split-screen login, sidebar dengan logo Dishub Surabaya, dan palet warna konsisten</t>
+  </si>
+  <si>
+    <t>Implementasi Backend (API)</t>
+  </si>
+  <si>
+    <t>REST API Laravel 11 dengan autentikasi Sanctum dan middleware role-based</t>
+  </si>
+  <si>
+    <t>Semua endpoint berfungsi untuk 3 role (Applicant, Admin, Head)</t>
+  </si>
+  <si>
+    <t>15+ endpoint API berfungsi termasuk algoritma DSS, CRUD divisi, dan export</t>
+  </si>
+  <si>
+    <t>Implementasi Frontend</t>
+  </si>
+  <si>
+    <t>Next.js 14 App Router dengan komponen reusable dan state management</t>
+  </si>
+  <si>
+    <t>Antarmuka responsif untuk semua role dengan navigasi yang intuitif</t>
+  </si>
+  <si>
+    <t>Komponen UI (Modal, Card, Button, Sidebar) bersifat reusable</t>
+  </si>
+  <si>
+    <t>Implementasi Database</t>
+  </si>
+  <si>
+    <t>PostgreSQL dengan 7 tabel utama dan relasi foreign key</t>
+  </si>
+  <si>
+    <t>Skema database mendukung seluruh fitur bisnis</t>
+  </si>
+  <si>
+    <t>Tabel: users, divisions, applications, documents, notifications, messages, export_logs</t>
+  </si>
+  <si>
+    <t>Implementasi File Storage</t>
+  </si>
+  <si>
+    <t>Supabase Storage untuk manajemen dokumen pelamar</t>
+  </si>
+  <si>
+    <t>Dokumen terunggah dan dapat diakses via Public URL</t>
+  </si>
+  <si>
+    <t>Upload dokumen berhasil, namun export Excel ke Supabase gagal (MIME type 415). Solusi: bypass Supabase untuk export</t>
+  </si>
+  <si>
+    <t>Fitur Preview Dokumen</t>
+  </si>
+  <si>
+    <t>Admin dapat mereview dokumen langsung di dalam aplikasi</t>
+  </si>
+  <si>
+    <t>Pop-up iframe menampilkan file PDF tanpa perlu download</t>
+  </si>
+  <si>
+    <t>Percobaan pertama gagal (404 error karena relative path). Setelah perbaikan Accessor URL, fitur berjalan normal</t>
+  </si>
+  <si>
+    <t>Fitur Algoritma DSS</t>
+  </si>
+  <si>
+    <t>Sistem mengevaluasi pelamar otomatis berdasarkan R1, R3, R4</t>
+  </si>
+  <si>
+    <t>Skor dan status evaluasi ditampilkan sebelum admin memutuskan</t>
+  </si>
+  <si>
+    <t>Tiga rule (Dokumen, Kuota, Keyword Matching) berfungsi dengan threshold skor 60</t>
+  </si>
+  <si>
+    <t>Fitur Export Laporan</t>
+  </si>
+  <si>
+    <t>Pimpinan dapat mengunduh laporan Excel dengan filter</t>
+  </si>
+  <si>
+    <t>File .xlsx terunduh otomatis sesuai filter yang dipilih</t>
+  </si>
+  <si>
+    <t>Gagal 2 kali (MIME type 415 + PHP return type error). Berhasil setelah perombakan arsitektur ke direct binary stream</t>
+  </si>
+  <si>
+    <t>Fitur Dashboard Analitik</t>
+  </si>
+  <si>
+    <t>Pimpinan melihat statistik lengkap dan dapat merefresh data</t>
+  </si>
+  <si>
+    <t>Dashboard menampilkan grafik, statistik, dan tombol refresh</t>
+  </si>
+  <si>
+    <t>Grafik Recharts, statistik real-time, dan tombol refresh manual berfungsi</t>
+  </si>
+  <si>
+    <t>Blackbox dan Whitebox testing pada seluruh fitur utama</t>
+  </si>
+  <si>
+    <t>Seluruh fitur lulus pengujian</t>
+  </si>
+  <si>
+    <t>3 dari 20 kasus Blackbox tidak lulus pada percobaan pertama (Preview 404, Export MIME 415, Export return type). Semua berhasil setelah perbaikan</t>
+  </si>
+  <si>
+    <t>Sistem berjalan di lingkungan lokal</t>
+  </si>
+  <si>
+    <t>Backend dan Frontend berjalan bersamaan tanpa konflik</t>
+  </si>
+  <si>
+    <t>Backend: localhost:8000, Frontend: localhost:3000 berjalan stabil</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -559,22 +1216,84 @@
       <color theme="1"/>
       <name val="Arial"/>
     </font>
+    <font>
+      <color theme="1"/>
+      <name val="Roboto"/>
+    </font>
+    <font>
+      <color rgb="FF11734B"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF6F8F9"/>
+        <bgColor rgb="FFF6F8F9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border/>
+    <border>
+      <left style="thin">
+        <color rgb="FFD1D5DB"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD1D5DB"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD1D5DB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD1D5DB"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFFFFFFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFF6F8F9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFF6F8F9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFF6F8F9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFF6F8F9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="28">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -631,6 +1350,30 @@
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="2" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="3" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -692,7 +1435,7 @@
       </border>
     </dxf>
   </dxfs>
-  <tableStyles count="8">
+  <tableStyles count="11">
     <tableStyle count="4" pivot="0" name="Contoh_Objektivitas-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
@@ -724,6 +1467,24 @@
       <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
     </tableStyle>
     <tableStyle count="4" pivot="0" name="BlackBox-style">
+      <tableStyleElement dxfId="1" type="headerRow"/>
+      <tableStyleElement dxfId="2" type="firstRowStripe"/>
+      <tableStyleElement dxfId="3" type="secondRowStripe"/>
+      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    </tableStyle>
+    <tableStyle count="4" pivot="0" name="BlackBox-style 2">
+      <tableStyleElement dxfId="1" type="headerRow"/>
+      <tableStyleElement dxfId="2" type="firstRowStripe"/>
+      <tableStyleElement dxfId="3" type="secondRowStripe"/>
+      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    </tableStyle>
+    <tableStyle count="4" pivot="0" name="BlackBox-style 3">
+      <tableStyleElement dxfId="1" type="headerRow"/>
+      <tableStyleElement dxfId="2" type="firstRowStripe"/>
+      <tableStyleElement dxfId="3" type="secondRowStripe"/>
+      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    </tableStyle>
+    <tableStyle count="4" pivot="0" name="BlackBox-style 4">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
@@ -792,6 +1553,36 @@
 </table>
 </file>
 
+<file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:I11" displayName="Pengujian_Whitebox" name="Pengujian_Whitebox" id="10">
+  <tableColumns count="9">
+    <tableColumn name="ID Kasus Uji" id="1"/>
+    <tableColumn name="Skenario Uji" id="2"/>
+    <tableColumn name="Kode yang Diuji" id="3"/>
+    <tableColumn name="Data Masukan" id="4"/>
+    <tableColumn name="Hasil yang Diharapkan" id="5"/>
+    <tableColumn name="Hasil Aktual" id="6"/>
+    <tableColumn name="Cakupan Kode" id="7"/>
+    <tableColumn name="Status (Lulus/Tidak Lulus)" id="8"/>
+    <tableColumn name="Catatan" id="9"/>
+  </tableColumns>
+  <tableStyleInfo name="WhiteBox-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E18" displayName="HasilCapaian" name="HasilCapaian" id="11">
+  <tableColumns count="5">
+    <tableColumn name="Objektivitas" id="1"/>
+    <tableColumn name="Target (Disesuaikan dengan Kondisi Kelompok)*" id="2"/>
+    <tableColumn name="Ekspektasi" id="3"/>
+    <tableColumn name="Status (Sesuai/Tidak Sesuai)" id="4"/>
+    <tableColumn name="Catatan" id="5"/>
+  </tableColumns>
+  <tableStyleInfo name="Hasil Capaian-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:G12" displayName="Contoh_BlackBox" name="Contoh_BlackBox" id="2">
   <tableColumns count="7">
@@ -839,17 +1630,18 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:B18" displayName="SesuaiMetodeKelompok" name="SesuaiMetodeKelompok" id="5">
-  <tableColumns count="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:C18" displayName="SesuaiMetodeKelompok" name="SesuaiMetodeKelompok" id="5">
+  <tableColumns count="3">
     <tableColumn name="Objektivitas" id="1"/>
-    <tableColumn name="Target (Disesuaikan dengan Kondisi Kelompok)" id="2"/>
+    <tableColumn name="Metode" id="2"/>
+    <tableColumn name="Target (Disesuaikan dengan Kondisi Kelompok)" id="3"/>
   </tableColumns>
   <tableStyleInfo name="Objektivitas-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:G12" displayName="Table1" name="Table1" id="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:G5" displayName="Login_Register" name="Login_Register" id="6">
   <tableColumns count="7">
     <tableColumn name="ID Kasus Uji" id="1"/>
     <tableColumn name="Skenario Uji" id="2"/>
@@ -864,32 +1656,47 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:I7" displayName="Table2" name="Table2" id="7">
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A8:G11" displayName="Pengajuan_Pelamar" name="Pengajuan_Pelamar" id="7">
+  <tableColumns count="7">
     <tableColumn name="ID Kasus Uji" id="1"/>
     <tableColumn name="Skenario Uji" id="2"/>
-    <tableColumn name="Kode yang Diuji" id="3"/>
-    <tableColumn name="Data Masukan" id="4"/>
-    <tableColumn name="Hasil yang Diharapkan" id="5"/>
-    <tableColumn name="Hasil Aktual" id="6"/>
-    <tableColumn name="Cakupan Kode" id="7"/>
-    <tableColumn name="Status (Lulus/Tidak Lulus)" id="8"/>
-    <tableColumn name="Catatan" id="9"/>
+    <tableColumn name="Data Masukan" id="3"/>
+    <tableColumn name="Hasil yang Diharapkan" id="4"/>
+    <tableColumn name="Hasil Aktual" id="5"/>
+    <tableColumn name="Status (Lulus/Tidak Lulus)" id="6"/>
+    <tableColumn name="Catatan" id="7"/>
   </tableColumns>
-  <tableStyleInfo name="WhiteBox-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="BlackBox-style 2" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:E18" displayName="HasilCapaian" name="HasilCapaian" id="8">
-  <tableColumns count="5">
-    <tableColumn name="Objektivitas" id="1"/>
-    <tableColumn name="Target (Disesuaikan dengan Kondisi Kelompok)*" id="2"/>
-    <tableColumn name="Ekspektasi" id="3"/>
-    <tableColumn name="Status (Sesuai/Tidak Sesuai)" id="4"/>
-    <tableColumn name="Catatan" id="5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A14:G21" displayName="Akses_Admin" name="Akses_Admin" id="8">
+  <tableColumns count="7">
+    <tableColumn name="ID Kasus Uji" id="1"/>
+    <tableColumn name="Skenario Uji" id="2"/>
+    <tableColumn name="Data Masukan" id="3"/>
+    <tableColumn name="Hasil yang Diharapkan" id="4"/>
+    <tableColumn name="Hasil Aktual" id="5"/>
+    <tableColumn name="Status (Lulus/Tidak Lulus)" id="6"/>
+    <tableColumn name="Catatan" id="7"/>
   </tableColumns>
-  <tableStyleInfo name="Hasil Capaian-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="BlackBox-style 3" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A24:G30" displayName="Akses_Pimpinan" name="Akses_Pimpinan" id="9">
+  <tableColumns count="7">
+    <tableColumn name="ID Kasus Uji" id="1"/>
+    <tableColumn name="Skenario Uji" id="2"/>
+    <tableColumn name="Data Masukan" id="3"/>
+    <tableColumn name="Hasil yang Diharapkan" id="4"/>
+    <tableColumn name="Hasil Aktual" id="5"/>
+    <tableColumn name="Status (Lulus/Tidak Lulus)" id="6"/>
+    <tableColumn name="Catatan" id="7"/>
+  </tableColumns>
+  <tableStyleInfo name="BlackBox-style 4" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
 </file>
 
@@ -18936,7 +19743,8 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
     <col customWidth="1" min="1" max="1" width="35.75"/>
-    <col customWidth="1" min="2" max="2" width="84.25"/>
+    <col customWidth="1" min="2" max="2" width="15.5"/>
+    <col customWidth="1" min="3" max="3" width="67.0"/>
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
@@ -18944,76 +19752,132 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
-      <c r="A2" s="2"/>
-      <c r="B2" s="3"/>
+      <c r="A2" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>172</v>
+      </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
-      <c r="A3" s="2"/>
-      <c r="B3" s="5"/>
+      <c r="A3" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>173</v>
+      </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="2"/>
-      <c r="B4" s="5"/>
+      <c r="A4" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="2"/>
-      <c r="B5" s="5"/>
+      <c r="A5" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>175</v>
+      </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="2"/>
-      <c r="B6" s="5"/>
+      <c r="A6" s="20" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>176</v>
+      </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="2"/>
-      <c r="B7" s="5"/>
+      <c r="A7" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>177</v>
+      </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="2"/>
-      <c r="B8" s="5"/>
+      <c r="A8" s="22"/>
+      <c r="B8" s="23"/>
+      <c r="C8" s="23"/>
     </row>
     <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="2"/>
-      <c r="B9" s="5"/>
+      <c r="A9" s="22"/>
+      <c r="B9" s="23"/>
+      <c r="C9" s="23"/>
     </row>
     <row r="10" ht="22.5" customHeight="1">
-      <c r="A10" s="2"/>
-      <c r="B10" s="5"/>
+      <c r="A10" s="22"/>
+      <c r="B10" s="23"/>
+      <c r="C10" s="23"/>
     </row>
     <row r="11" ht="22.5" customHeight="1">
-      <c r="A11" s="2"/>
-      <c r="B11" s="5"/>
+      <c r="A11" s="22"/>
+      <c r="B11" s="23"/>
+      <c r="C11" s="23"/>
     </row>
     <row r="12" ht="22.5" customHeight="1">
-      <c r="A12" s="2"/>
-      <c r="B12" s="5"/>
+      <c r="A12" s="22"/>
+      <c r="B12" s="23"/>
+      <c r="C12" s="23"/>
     </row>
     <row r="13" ht="22.5" customHeight="1">
-      <c r="A13" s="2"/>
-      <c r="B13" s="5"/>
+      <c r="A13" s="22"/>
+      <c r="B13" s="23"/>
+      <c r="C13" s="23"/>
     </row>
     <row r="14" ht="22.5" customHeight="1">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
+      <c r="A14" s="22"/>
+      <c r="B14" s="22"/>
+      <c r="C14" s="22"/>
     </row>
     <row r="15" ht="22.5" customHeight="1">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
+      <c r="A15" s="23"/>
+      <c r="B15" s="23"/>
+      <c r="C15" s="23"/>
     </row>
     <row r="16" ht="22.5" customHeight="1">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5"/>
+      <c r="A16" s="23"/>
+      <c r="B16" s="23"/>
+      <c r="C16" s="23"/>
     </row>
     <row r="17" ht="22.5" customHeight="1">
-      <c r="A17" s="5"/>
-      <c r="B17" s="5"/>
+      <c r="A17" s="23"/>
+      <c r="B17" s="23"/>
+      <c r="C17" s="23"/>
     </row>
     <row r="18" ht="22.5" customHeight="1">
-      <c r="A18" s="5"/>
-      <c r="B18" s="5"/>
+      <c r="A18" s="23"/>
+      <c r="B18" s="23"/>
+      <c r="C18" s="23"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>
@@ -19050,7 +19914,7 @@
         <v>38</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="E1" s="7" t="s">
         <v>40</v>
@@ -19063,134 +19927,384 @@
       </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
-      <c r="A2" s="3"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
+      <c r="A2" s="21" t="s">
+        <v>179</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>180</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>181</v>
+      </c>
+      <c r="D2" s="20" t="s">
+        <v>182</v>
+      </c>
+      <c r="E2" s="20" t="s">
+        <v>182</v>
+      </c>
       <c r="F2" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="8"/>
+      <c r="G2" s="20" t="s">
+        <v>183</v>
+      </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
-      <c r="A3" s="3"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="G3" s="8"/>
+      <c r="A3" s="21" t="s">
+        <v>184</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>185</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>186</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>187</v>
+      </c>
+      <c r="E3" s="20" t="s">
+        <v>187</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="G3" s="20" t="s">
+        <v>188</v>
+      </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="3"/>
-      <c r="B4" s="8"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="8"/>
+      <c r="A4" s="21" t="s">
+        <v>189</v>
+      </c>
+      <c r="B4" s="20" t="s">
+        <v>190</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>191</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>192</v>
+      </c>
+      <c r="E4" s="20" t="s">
+        <v>192</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="G4" s="20" t="s">
+        <v>193</v>
+      </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="3"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="8"/>
-    </row>
-    <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="3"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="8"/>
-    </row>
-    <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="3"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="8"/>
+      <c r="A5" s="21" t="s">
+        <v>194</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>195</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>196</v>
+      </c>
+      <c r="D5" s="20" t="s">
+        <v>197</v>
+      </c>
+      <c r="E5" s="20" t="s">
+        <v>197</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="G5" s="20" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="4"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="4"/>
     </row>
     <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="3"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="8"/>
+      <c r="A8" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="3"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="8"/>
+      <c r="A9" s="21" t="s">
+        <v>199</v>
+      </c>
+      <c r="B9" s="20" t="s">
+        <v>200</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>201</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>202</v>
+      </c>
+      <c r="E9" s="20" t="s">
+        <v>202</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="G9" s="20" t="s">
+        <v>203</v>
+      </c>
     </row>
     <row r="10" ht="22.5" customHeight="1">
-      <c r="A10" s="3"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="8"/>
+      <c r="A10" s="21" t="s">
+        <v>204</v>
+      </c>
+      <c r="B10" s="20" t="s">
+        <v>205</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>206</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>207</v>
+      </c>
+      <c r="E10" s="20" t="s">
+        <v>208</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="G10" s="20" t="s">
+        <v>209</v>
+      </c>
     </row>
     <row r="11" ht="22.5" customHeight="1">
-      <c r="A11" s="3"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="8"/>
-    </row>
-    <row r="12" ht="22.5" customHeight="1">
-      <c r="A12" s="2"/>
-      <c r="B12" s="12"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="12"/>
+      <c r="A11" s="21" t="s">
+        <v>210</v>
+      </c>
+      <c r="B11" s="20" t="s">
+        <v>211</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>212</v>
+      </c>
+      <c r="D11" s="20" t="s">
+        <v>213</v>
+      </c>
+      <c r="E11" s="20" t="s">
+        <v>213</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="G11" s="20" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="4"/>
     </row>
     <row r="13">
       <c r="B13" s="4"/>
     </row>
-    <row r="14">
-      <c r="B14" s="4"/>
-    </row>
-    <row r="15">
-      <c r="B15" s="4"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="4"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="4"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="4"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="4"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="4"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="4"/>
+    <row r="14" ht="22.5" customHeight="1">
+      <c r="A14" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G14" s="7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" ht="22.5" customHeight="1">
+      <c r="A15" s="21" t="s">
+        <v>215</v>
+      </c>
+      <c r="B15" s="20" t="s">
+        <v>216</v>
+      </c>
+      <c r="C15" s="20" t="s">
+        <v>217</v>
+      </c>
+      <c r="D15" s="20" t="s">
+        <v>218</v>
+      </c>
+      <c r="E15" s="20" t="s">
+        <v>218</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="G15" s="20" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="16" ht="22.5" customHeight="1">
+      <c r="A16" s="21" t="s">
+        <v>220</v>
+      </c>
+      <c r="B16" s="20" t="s">
+        <v>221</v>
+      </c>
+      <c r="C16" s="20" t="s">
+        <v>222</v>
+      </c>
+      <c r="D16" s="20" t="s">
+        <v>223</v>
+      </c>
+      <c r="E16" s="20" t="s">
+        <v>223</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="G16" s="20" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="17" ht="22.5" customHeight="1">
+      <c r="A17" s="21" t="s">
+        <v>225</v>
+      </c>
+      <c r="B17" s="20" t="s">
+        <v>226</v>
+      </c>
+      <c r="C17" s="20" t="s">
+        <v>227</v>
+      </c>
+      <c r="D17" s="20" t="s">
+        <v>228</v>
+      </c>
+      <c r="E17" s="20" t="s">
+        <v>228</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="G17" s="20" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="18" ht="22.5" customHeight="1">
+      <c r="A18" s="21" t="s">
+        <v>230</v>
+      </c>
+      <c r="B18" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="C18" s="20" t="s">
+        <v>232</v>
+      </c>
+      <c r="D18" s="20" t="s">
+        <v>233</v>
+      </c>
+      <c r="E18" s="20" t="s">
+        <v>234</v>
+      </c>
+      <c r="F18" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G18" s="20" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="19" ht="22.5" customHeight="1">
+      <c r="A19" s="21" t="s">
+        <v>236</v>
+      </c>
+      <c r="B19" s="20" t="s">
+        <v>237</v>
+      </c>
+      <c r="C19" s="20" t="s">
+        <v>232</v>
+      </c>
+      <c r="D19" s="20" t="s">
+        <v>233</v>
+      </c>
+      <c r="E19" s="20" t="s">
+        <v>238</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="G19" s="20" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="20" ht="22.5" customHeight="1">
+      <c r="A20" s="21" t="s">
+        <v>240</v>
+      </c>
+      <c r="B20" s="20" t="s">
+        <v>241</v>
+      </c>
+      <c r="C20" s="20" t="s">
+        <v>242</v>
+      </c>
+      <c r="D20" s="20" t="s">
+        <v>243</v>
+      </c>
+      <c r="E20" s="20" t="s">
+        <v>243</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="G20" s="20" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="21" ht="22.5" customHeight="1">
+      <c r="A21" s="21" t="s">
+        <v>245</v>
+      </c>
+      <c r="B21" s="20" t="s">
+        <v>246</v>
+      </c>
+      <c r="C21" s="20" t="s">
+        <v>247</v>
+      </c>
+      <c r="D21" s="20" t="s">
+        <v>248</v>
+      </c>
+      <c r="E21" s="20" t="s">
+        <v>248</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="G21" s="20" t="s">
+        <v>249</v>
+      </c>
     </row>
     <row r="22">
       <c r="B22" s="4"/>
@@ -19198,26 +20312,166 @@
     <row r="23">
       <c r="B23" s="4"/>
     </row>
-    <row r="24">
-      <c r="B24" s="4"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="4"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="4"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="4"/>
-    </row>
-    <row r="28">
-      <c r="B28" s="4"/>
-    </row>
-    <row r="29">
-      <c r="B29" s="4"/>
-    </row>
-    <row r="30">
-      <c r="B30" s="4"/>
+    <row r="24" ht="22.5" customHeight="1">
+      <c r="A24" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" ht="22.5" customHeight="1">
+      <c r="A25" s="21" t="s">
+        <v>250</v>
+      </c>
+      <c r="B25" s="20" t="s">
+        <v>251</v>
+      </c>
+      <c r="C25" s="20" t="s">
+        <v>252</v>
+      </c>
+      <c r="D25" s="20" t="s">
+        <v>253</v>
+      </c>
+      <c r="E25" s="20" t="s">
+        <v>253</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="G25" s="20" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="26" ht="22.5" customHeight="1">
+      <c r="A26" s="21" t="s">
+        <v>255</v>
+      </c>
+      <c r="B26" s="20" t="s">
+        <v>256</v>
+      </c>
+      <c r="C26" s="20" t="s">
+        <v>257</v>
+      </c>
+      <c r="D26" s="20" t="s">
+        <v>258</v>
+      </c>
+      <c r="E26" s="20" t="s">
+        <v>259</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="G26" s="20" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="27" ht="22.5" customHeight="1">
+      <c r="A27" s="21" t="s">
+        <v>261</v>
+      </c>
+      <c r="B27" s="20" t="s">
+        <v>262</v>
+      </c>
+      <c r="C27" s="20" t="s">
+        <v>263</v>
+      </c>
+      <c r="D27" s="20" t="s">
+        <v>264</v>
+      </c>
+      <c r="E27" s="20" t="s">
+        <v>265</v>
+      </c>
+      <c r="F27" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G27" s="20" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="28" ht="22.5" customHeight="1">
+      <c r="A28" s="21" t="s">
+        <v>267</v>
+      </c>
+      <c r="B28" s="20" t="s">
+        <v>268</v>
+      </c>
+      <c r="C28" s="20" t="s">
+        <v>269</v>
+      </c>
+      <c r="D28" s="20" t="s">
+        <v>264</v>
+      </c>
+      <c r="E28" s="20" t="s">
+        <v>270</v>
+      </c>
+      <c r="F28" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G28" s="20" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="29" ht="22.5" customHeight="1">
+      <c r="A29" s="21" t="s">
+        <v>272</v>
+      </c>
+      <c r="B29" s="20" t="s">
+        <v>273</v>
+      </c>
+      <c r="C29" s="20" t="s">
+        <v>263</v>
+      </c>
+      <c r="D29" s="20" t="s">
+        <v>264</v>
+      </c>
+      <c r="E29" s="20" t="s">
+        <v>274</v>
+      </c>
+      <c r="F29" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="G29" s="20" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="30" ht="22.5" customHeight="1">
+      <c r="A30" s="21" t="s">
+        <v>276</v>
+      </c>
+      <c r="B30" s="20" t="s">
+        <v>277</v>
+      </c>
+      <c r="C30" s="20" t="s">
+        <v>278</v>
+      </c>
+      <c r="D30" s="20" t="s">
+        <v>279</v>
+      </c>
+      <c r="E30" s="20" t="s">
+        <v>280</v>
+      </c>
+      <c r="F30" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="G30" s="20" t="s">
+        <v>281</v>
+      </c>
     </row>
     <row r="31">
       <c r="B31" s="4"/>
@@ -22078,66 +23332,18 @@
     <row r="983">
       <c r="B983" s="4"/>
     </row>
-    <row r="984">
-      <c r="B984" s="4"/>
-    </row>
-    <row r="985">
-      <c r="B985" s="4"/>
-    </row>
-    <row r="986">
-      <c r="B986" s="4"/>
-    </row>
-    <row r="987">
-      <c r="B987" s="4"/>
-    </row>
-    <row r="988">
-      <c r="B988" s="4"/>
-    </row>
-    <row r="989">
-      <c r="B989" s="4"/>
-    </row>
-    <row r="990">
-      <c r="B990" s="4"/>
-    </row>
-    <row r="991">
-      <c r="B991" s="4"/>
-    </row>
-    <row r="992">
-      <c r="B992" s="4"/>
-    </row>
-    <row r="993">
-      <c r="B993" s="4"/>
-    </row>
-    <row r="994">
-      <c r="B994" s="4"/>
-    </row>
-    <row r="995">
-      <c r="B995" s="4"/>
-    </row>
-    <row r="996">
-      <c r="B996" s="4"/>
-    </row>
-    <row r="997">
-      <c r="B997" s="4"/>
-    </row>
-    <row r="998">
-      <c r="B998" s="4"/>
-    </row>
-    <row r="999">
-      <c r="B999" s="4"/>
-    </row>
-    <row r="1000">
-      <c r="B1000" s="4"/>
-    </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="F2:F12">
+    <dataValidation type="list" allowBlank="1" sqref="F2:F5 F9:F11 F15:F21 F25:F30">
       <formula1>"Lulus,Tidak Lulus"</formula1>
     </dataValidation>
   </dataValidations>
   <drawing r:id="rId1"/>
-  <tableParts count="1">
-    <tablePart r:id="rId3"/>
+  <tableParts count="4">
+    <tablePart r:id="rId6"/>
+    <tablePart r:id="rId7"/>
+    <tablePart r:id="rId8"/>
+    <tablePart r:id="rId9"/>
   </tableParts>
 </worksheet>
 </file>
@@ -22151,7 +23357,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="14.38"/>
     <col customWidth="1" min="2" max="2" width="31.75"/>
-    <col customWidth="1" min="3" max="3" width="20.75"/>
+    <col customWidth="1" min="3" max="3" width="20.88"/>
     <col customWidth="1" min="4" max="4" width="25.88"/>
     <col customWidth="1" min="5" max="5" width="24.5"/>
     <col customWidth="1" min="6" max="6" width="31.75"/>
@@ -22172,7 +23378,7 @@
         <v>38</v>
       </c>
       <c r="E1" s="7" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="F1" s="7" t="s">
         <v>40</v>
@@ -22188,182 +23394,298 @@
       </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="24" t="s">
         <v>106</v>
       </c>
-      <c r="B2" s="15" t="s">
-        <v>107</v>
-      </c>
-      <c r="C2" s="15" t="s">
-        <v>108</v>
-      </c>
-      <c r="D2" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="E2" s="15" t="s">
-        <v>109</v>
-      </c>
-      <c r="F2" s="15" t="s">
-        <v>110</v>
-      </c>
-      <c r="G2" s="15" t="s">
-        <v>111</v>
+      <c r="B2" s="25" t="s">
+        <v>282</v>
+      </c>
+      <c r="C2" s="25" t="s">
+        <v>283</v>
+      </c>
+      <c r="D2" s="25" t="s">
+        <v>284</v>
+      </c>
+      <c r="E2" s="25" t="s">
+        <v>285</v>
+      </c>
+      <c r="F2" s="25" t="s">
+        <v>286</v>
+      </c>
+      <c r="G2" s="25" t="s">
+        <v>287</v>
       </c>
       <c r="H2" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="I2" s="15" t="s">
-        <v>112</v>
+      <c r="I2" s="25" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="24" t="s">
         <v>113</v>
       </c>
-      <c r="B3" s="15" t="s">
-        <v>114</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>108</v>
-      </c>
-      <c r="D3" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="E3" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="F3" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="G3" s="15" t="s">
-        <v>116</v>
+      <c r="B3" s="25" t="s">
+        <v>289</v>
+      </c>
+      <c r="C3" s="25" t="s">
+        <v>283</v>
+      </c>
+      <c r="D3" s="25" t="s">
+        <v>290</v>
+      </c>
+      <c r="E3" s="25" t="s">
+        <v>291</v>
+      </c>
+      <c r="F3" s="25" t="s">
+        <v>291</v>
+      </c>
+      <c r="G3" s="25" t="s">
+        <v>292</v>
       </c>
       <c r="H3" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="I3" s="15" t="s">
-        <v>117</v>
+      <c r="I3" s="25" t="s">
+        <v>293</v>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="24" t="s">
         <v>118</v>
       </c>
-      <c r="B4" s="15" t="s">
-        <v>119</v>
-      </c>
-      <c r="C4" s="15" t="s">
-        <v>120</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="E4" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="F4" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="G4" s="15" t="s">
-        <v>124</v>
+      <c r="B4" s="25" t="s">
+        <v>294</v>
+      </c>
+      <c r="C4" s="25" t="s">
+        <v>283</v>
+      </c>
+      <c r="D4" s="25" t="s">
+        <v>295</v>
+      </c>
+      <c r="E4" s="25" t="s">
+        <v>296</v>
+      </c>
+      <c r="F4" s="25" t="s">
+        <v>296</v>
+      </c>
+      <c r="G4" s="25" t="s">
+        <v>297</v>
       </c>
       <c r="H4" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="I4" s="15" t="s">
-        <v>125</v>
+      <c r="I4" s="25" t="s">
+        <v>298</v>
       </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="24" t="s">
         <v>126</v>
       </c>
-      <c r="B5" s="15" t="s">
-        <v>127</v>
-      </c>
-      <c r="C5" s="15" t="s">
-        <v>128</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="E5" s="15" t="s">
-        <v>130</v>
-      </c>
-      <c r="F5" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="G5" s="15" t="s">
-        <v>132</v>
-      </c>
-      <c r="H5" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="I5" s="15" t="s">
-        <v>133</v>
+      <c r="B5" s="25" t="s">
+        <v>299</v>
+      </c>
+      <c r="C5" s="25" t="s">
+        <v>300</v>
+      </c>
+      <c r="D5" s="25" t="s">
+        <v>301</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>302</v>
+      </c>
+      <c r="F5" s="25" t="s">
+        <v>303</v>
+      </c>
+      <c r="G5" s="25" t="s">
+        <v>304</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="I5" s="25" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="24" t="s">
         <v>134</v>
       </c>
-      <c r="B6" s="15" t="s">
-        <v>135</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>137</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>138</v>
-      </c>
-      <c r="F6" s="15" t="s">
-        <v>139</v>
-      </c>
-      <c r="G6" s="15" t="s">
-        <v>140</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="I6" s="15" t="s">
-        <v>141</v>
+      <c r="B6" s="25" t="s">
+        <v>306</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>307</v>
+      </c>
+      <c r="D6" s="25" t="s">
+        <v>301</v>
+      </c>
+      <c r="E6" s="25" t="s">
+        <v>308</v>
+      </c>
+      <c r="F6" s="25" t="s">
+        <v>309</v>
+      </c>
+      <c r="G6" s="25" t="s">
+        <v>310</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="I6" s="25" t="s">
+        <v>311</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="24" t="s">
         <v>142</v>
       </c>
-      <c r="B7" s="16" t="s">
-        <v>143</v>
-      </c>
-      <c r="C7" s="16" t="s">
-        <v>128</v>
-      </c>
-      <c r="D7" s="16" t="s">
-        <v>144</v>
-      </c>
-      <c r="E7" s="16" t="s">
-        <v>145</v>
-      </c>
-      <c r="F7" s="16" t="s">
-        <v>146</v>
-      </c>
-      <c r="G7" s="15" t="s">
-        <v>140</v>
+      <c r="B7" s="25" t="s">
+        <v>312</v>
+      </c>
+      <c r="C7" s="25" t="s">
+        <v>313</v>
+      </c>
+      <c r="D7" s="25" t="s">
+        <v>301</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>314</v>
+      </c>
+      <c r="F7" s="25" t="s">
+        <v>315</v>
+      </c>
+      <c r="G7" s="25" t="s">
+        <v>316</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="I7" s="16" t="s">
-        <v>147</v>
+      <c r="I7" s="25" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="8" ht="22.5" customHeight="1">
+      <c r="A8" s="24" t="s">
+        <v>318</v>
+      </c>
+      <c r="B8" s="25" t="s">
+        <v>319</v>
+      </c>
+      <c r="C8" s="25" t="s">
+        <v>320</v>
+      </c>
+      <c r="D8" s="25" t="s">
+        <v>321</v>
+      </c>
+      <c r="E8" s="25" t="s">
+        <v>322</v>
+      </c>
+      <c r="F8" s="25" t="s">
+        <v>322</v>
+      </c>
+      <c r="G8" s="25" t="s">
+        <v>323</v>
+      </c>
+      <c r="H8" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="I8" s="25" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="9" ht="22.5" customHeight="1">
+      <c r="A9" s="24" t="s">
+        <v>325</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>326</v>
+      </c>
+      <c r="C9" s="25" t="s">
+        <v>327</v>
+      </c>
+      <c r="D9" s="25" t="s">
+        <v>328</v>
+      </c>
+      <c r="E9" s="25" t="s">
+        <v>329</v>
+      </c>
+      <c r="F9" s="25" t="s">
+        <v>330</v>
+      </c>
+      <c r="G9" s="25" t="s">
+        <v>331</v>
+      </c>
+      <c r="H9" s="27" t="s">
+        <v>48</v>
+      </c>
+      <c r="I9" s="25" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="10" ht="22.5" customHeight="1">
+      <c r="A10" s="24" t="s">
+        <v>333</v>
+      </c>
+      <c r="B10" s="25" t="s">
+        <v>334</v>
+      </c>
+      <c r="C10" s="25" t="s">
+        <v>335</v>
+      </c>
+      <c r="D10" s="25" t="s">
+        <v>336</v>
+      </c>
+      <c r="E10" s="25" t="s">
+        <v>337</v>
+      </c>
+      <c r="F10" s="25" t="s">
+        <v>338</v>
+      </c>
+      <c r="G10" s="25" t="s">
+        <v>339</v>
+      </c>
+      <c r="H10" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="I10" s="25" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="11" ht="22.5" customHeight="1">
+      <c r="A11" s="24" t="s">
+        <v>341</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>342</v>
+      </c>
+      <c r="C11" s="25" t="s">
+        <v>343</v>
+      </c>
+      <c r="D11" s="25" t="s">
+        <v>344</v>
+      </c>
+      <c r="E11" s="25" t="s">
+        <v>345</v>
+      </c>
+      <c r="F11" s="25" t="s">
+        <v>345</v>
+      </c>
+      <c r="G11" s="25" t="s">
+        <v>346</v>
+      </c>
+      <c r="H11" s="26" t="s">
+        <v>48</v>
+      </c>
+      <c r="I11" s="25" t="s">
+        <v>347</v>
       </c>
     </row>
   </sheetData>
   <dataValidations>
-    <dataValidation type="list" allowBlank="1" sqref="H2:H7">
+    <dataValidation type="list" allowBlank="1" sqref="H2:H11">
       <formula1>"Lulus,Tidak Lulus"</formula1>
     </dataValidation>
   </dataValidations>
@@ -22385,6 +23707,7 @@
     <col customWidth="1" min="2" max="2" width="50.0"/>
     <col customWidth="1" min="3" max="3" width="37.25"/>
     <col customWidth="1" min="4" max="4" width="14.25"/>
+    <col customWidth="1" min="5" max="5" width="45.63"/>
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
@@ -22405,14 +23728,20 @@
       </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
-      <c r="A2" s="12"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
+      <c r="A2" s="25" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="25" t="s">
+        <v>348</v>
+      </c>
+      <c r="C2" s="25" t="s">
+        <v>349</v>
+      </c>
       <c r="D2" s="13" t="s">
         <v>151</v>
       </c>
-      <c r="E2" s="8" t="s">
-        <v>152</v>
+      <c r="E2" s="25" t="s">
+        <v>350</v>
       </c>
       <c r="F2" s="4"/>
       <c r="G2" s="4"/>
@@ -22442,14 +23771,20 @@
       <c r="AE2" s="4"/>
     </row>
     <row r="3" ht="22.5" customHeight="1">
-      <c r="A3" s="12"/>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
+      <c r="A3" s="25" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="25" t="s">
+        <v>351</v>
+      </c>
+      <c r="C3" s="25" t="s">
+        <v>352</v>
+      </c>
       <c r="D3" s="13" t="s">
         <v>154</v>
       </c>
-      <c r="E3" s="8" t="s">
-        <v>152</v>
+      <c r="E3" s="25" t="s">
+        <v>353</v>
       </c>
       <c r="F3" s="6"/>
       <c r="G3" s="6"/>
@@ -22479,11 +23814,21 @@
       <c r="AE3" s="4"/>
     </row>
     <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="12"/>
-      <c r="B4" s="19"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="8"/>
+      <c r="A4" s="25" t="s">
+        <v>354</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>355</v>
+      </c>
+      <c r="C4" s="25" t="s">
+        <v>356</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="E4" s="25" t="s">
+        <v>357</v>
+      </c>
       <c r="F4" s="6"/>
       <c r="G4" s="6"/>
       <c r="H4" s="6"/>
@@ -22512,11 +23857,21 @@
       <c r="AE4" s="4"/>
     </row>
     <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="12"/>
-      <c r="B5" s="19"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="8"/>
+      <c r="A5" s="25" t="s">
+        <v>358</v>
+      </c>
+      <c r="B5" s="25" t="s">
+        <v>359</v>
+      </c>
+      <c r="C5" s="25" t="s">
+        <v>360</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="E5" s="25" t="s">
+        <v>361</v>
+      </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
@@ -22545,11 +23900,21 @@
       <c r="AE5" s="4"/>
     </row>
     <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="12"/>
-      <c r="B6" s="19"/>
-      <c r="C6" s="19"/>
-      <c r="D6" s="13"/>
-      <c r="E6" s="8"/>
+      <c r="A6" s="25" t="s">
+        <v>362</v>
+      </c>
+      <c r="B6" s="25" t="s">
+        <v>363</v>
+      </c>
+      <c r="C6" s="25" t="s">
+        <v>364</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="E6" s="25" t="s">
+        <v>365</v>
+      </c>
       <c r="F6" s="6"/>
       <c r="G6" s="6"/>
       <c r="H6" s="6"/>
@@ -22578,11 +23943,21 @@
       <c r="AE6" s="4"/>
     </row>
     <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="12"/>
-      <c r="B7" s="19"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="8"/>
+      <c r="A7" s="25" t="s">
+        <v>366</v>
+      </c>
+      <c r="B7" s="25" t="s">
+        <v>367</v>
+      </c>
+      <c r="C7" s="25" t="s">
+        <v>368</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="E7" s="25" t="s">
+        <v>369</v>
+      </c>
       <c r="F7" s="6"/>
       <c r="G7" s="6"/>
       <c r="H7" s="6"/>
@@ -22611,11 +23986,21 @@
       <c r="AE7" s="4"/>
     </row>
     <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="12"/>
-      <c r="B8" s="19"/>
-      <c r="C8" s="19"/>
-      <c r="D8" s="13"/>
-      <c r="E8" s="8"/>
+      <c r="A8" s="25" t="s">
+        <v>370</v>
+      </c>
+      <c r="B8" s="25" t="s">
+        <v>371</v>
+      </c>
+      <c r="C8" s="25" t="s">
+        <v>372</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="E8" s="25" t="s">
+        <v>373</v>
+      </c>
       <c r="F8" s="6"/>
       <c r="G8" s="6"/>
       <c r="H8" s="6"/>
@@ -22644,11 +24029,21 @@
       <c r="AE8" s="4"/>
     </row>
     <row r="9" ht="22.5" customHeight="1">
-      <c r="A9" s="12"/>
-      <c r="B9" s="19"/>
-      <c r="C9" s="19"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="8"/>
+      <c r="A9" s="25" t="s">
+        <v>374</v>
+      </c>
+      <c r="B9" s="25" t="s">
+        <v>375</v>
+      </c>
+      <c r="C9" s="25" t="s">
+        <v>376</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="E9" s="25" t="s">
+        <v>377</v>
+      </c>
       <c r="F9" s="6"/>
       <c r="G9" s="6"/>
       <c r="H9" s="6"/>
@@ -22677,11 +24072,21 @@
       <c r="AE9" s="4"/>
     </row>
     <row r="10" ht="22.5" customHeight="1">
-      <c r="A10" s="12"/>
-      <c r="B10" s="19"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="8"/>
+      <c r="A10" s="25" t="s">
+        <v>378</v>
+      </c>
+      <c r="B10" s="25" t="s">
+        <v>379</v>
+      </c>
+      <c r="C10" s="25" t="s">
+        <v>380</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="E10" s="25" t="s">
+        <v>381</v>
+      </c>
       <c r="F10" s="6"/>
       <c r="G10" s="6"/>
       <c r="H10" s="6"/>
@@ -22710,11 +24115,21 @@
       <c r="AE10" s="4"/>
     </row>
     <row r="11" ht="22.5" customHeight="1">
-      <c r="A11" s="12"/>
-      <c r="B11" s="19"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="8"/>
+      <c r="A11" s="25" t="s">
+        <v>382</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>383</v>
+      </c>
+      <c r="C11" s="25" t="s">
+        <v>384</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="E11" s="25" t="s">
+        <v>385</v>
+      </c>
       <c r="F11" s="6"/>
       <c r="G11" s="6"/>
       <c r="H11" s="6"/>
@@ -22743,11 +24158,21 @@
       <c r="AE11" s="4"/>
     </row>
     <row r="12" ht="22.5" customHeight="1">
-      <c r="A12" s="12"/>
-      <c r="B12" s="19"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="8"/>
+      <c r="A12" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12" s="25" t="s">
+        <v>386</v>
+      </c>
+      <c r="C12" s="25" t="s">
+        <v>387</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="E12" s="25" t="s">
+        <v>388</v>
+      </c>
       <c r="F12" s="6"/>
       <c r="G12" s="6"/>
       <c r="H12" s="6"/>
@@ -22776,11 +24201,21 @@
       <c r="AE12" s="4"/>
     </row>
     <row r="13" ht="22.5" customHeight="1">
-      <c r="A13" s="12"/>
-      <c r="B13" s="19"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="13"/>
-      <c r="E13" s="8"/>
+      <c r="A13" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>389</v>
+      </c>
+      <c r="C13" s="25" t="s">
+        <v>390</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="E13" s="25" t="s">
+        <v>391</v>
+      </c>
       <c r="F13" s="6"/>
       <c r="G13" s="6"/>
       <c r="H13" s="6"/>

</xml_diff>